<commit_message>
docs and results: reproduced numbers, add GUIDE, remove long dashes
</commit_message>
<xml_diff>
--- a/results/S4-Optimization.xlsx
+++ b/results/S4-Optimization.xlsx
@@ -2265,10 +2265,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="227" min="1" max="1"/>
+    <col width="16" customWidth="1" style="227" min="1" max="1"/>
     <col width="10" customWidth="1" style="227" min="2" max="2"/>
     <col width="18" customWidth="1" style="227" min="3" max="3"/>
     <col width="14" customWidth="1" style="227" min="4" max="4"/>
@@ -2281,14 +2281,14 @@
     <row r="1">
       <c r="A1" s="231" t="inlineStr">
         <is>
-          <t>Controlled experiment: d64 vs d108 at a FIXED sequence length (256)</t>
+          <t>Controlled experiment: d64 vs d108 at a FIXED sequence length (256), plus d64 native</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="232" t="inlineStr">
         <is>
-          <t>Both models use 256 tokens (4x4 patches), so the only variables are width and depth. Isolates model size from sequence length. RiscvMinorCPU, VLEN 256, 22 nm, fp 0.60, one inference.</t>
+          <t>Reproduced from a clean checkout. RiscvMinorCPU, VLEN 256, 22 nm, fp 0.60, one inference. Both seq256 models use 256 tokens; only width and depth differ.</t>
         </is>
       </c>
     </row>
@@ -2346,22 +2346,22 @@
         </is>
       </c>
       <c r="C5" s="236" t="n">
-        <v>6268591</v>
+        <v>6275503</v>
       </c>
       <c r="D5" s="237" t="n">
-        <v>0.08339000000000001</v>
+        <v>0.086399</v>
       </c>
       <c r="E5" s="238" t="n">
-        <v>0.0111675</v>
+        <v>0.0101353</v>
       </c>
       <c r="F5" s="239" t="n">
-        <v>0.9312578250000001</v>
+        <v>0.8756797847000001</v>
       </c>
       <c r="G5" s="239" t="n">
-        <v>11.99184554502938</v>
+        <v>11.57420803481522</v>
       </c>
       <c r="H5" s="239" t="n">
-        <v>0.07765759002675002</v>
+        <v>0.07565785771829531</v>
       </c>
     </row>
     <row r="6">
@@ -2376,22 +2376,22 @@
         </is>
       </c>
       <c r="C6" s="242" t="n">
-        <v>12475543</v>
+        <v>12468631</v>
       </c>
       <c r="D6" s="243" t="n">
-        <v>0.201427</v>
+        <v>0.201345</v>
       </c>
       <c r="E6" s="244" t="n">
-        <v>0.00958645</v>
+        <v>0.00868087</v>
       </c>
       <c r="F6" s="245" t="n">
-        <v>1.93096986415</v>
+        <v>1.74784977015</v>
       </c>
       <c r="G6" s="245" t="n">
-        <v>4.964577737840508</v>
+        <v>4.96659961757183</v>
       </c>
       <c r="H6" s="245" t="n">
-        <v>0.388949466826142</v>
+        <v>0.3519208119708517</v>
       </c>
     </row>
     <row r="7">
@@ -2409,19 +2409,19 @@
         <v>19948310</v>
       </c>
       <c r="D7" s="237" t="n">
-        <v>0.286467</v>
+        <v>0.287988</v>
       </c>
       <c r="E7" s="238" t="n">
-        <v>0.0105062</v>
+        <v>0.009919880000000001</v>
       </c>
       <c r="F7" s="239" t="n">
-        <v>3.009679595400001</v>
+        <v>2.856806401440001</v>
       </c>
       <c r="G7" s="239" t="n">
-        <v>3.490803478236586</v>
+        <v>3.472366904176563</v>
       </c>
       <c r="H7" s="239" t="n">
-        <v>0.8621738846554521</v>
+        <v>0.8227259619379029</v>
       </c>
     </row>
     <row r="8">
@@ -2442,182 +2442,181 @@
         <v>0.53195</v>
       </c>
       <c r="E8" s="244" t="n">
-        <v>0.00961045</v>
+        <v>0.0089739</v>
       </c>
       <c r="F8" s="245" t="n">
-        <v>5.112278877500001</v>
+        <v>4.773666105</v>
       </c>
       <c r="G8" s="245" t="n">
         <v>1.879875928188739</v>
       </c>
       <c r="H8" s="245" t="n">
-        <v>2.719476748886125</v>
+        <v>2.53935168455475</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="234" t="inlineStr">
+        <is>
+          <t>d64_native</t>
+        </is>
+      </c>
+      <c r="B9" s="235" t="inlineStr">
+        <is>
+          <t>RVV</t>
+        </is>
+      </c>
+      <c r="C9" s="236" t="n">
+        <v>58481032</v>
+      </c>
+      <c r="D9" s="237" t="n">
+        <v>0.715607</v>
+      </c>
+      <c r="E9" s="238" t="n">
+        <v>0.0113697</v>
+      </c>
+      <c r="F9" s="239" t="n">
+        <v>8.136236907899999</v>
+      </c>
+      <c r="G9" s="239" t="n">
+        <v>1.397415061619017</v>
+      </c>
+      <c r="H9" s="239" t="n">
+        <v>5.822348084951595</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="246" t="inlineStr">
-        <is>
-          <t>Controlled comparison at fixed sequence 256 (RVV builds)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="233" t="inlineStr">
+      <c r="A10" s="240" t="inlineStr">
+        <is>
+          <t>d64_native</t>
+        </is>
+      </c>
+      <c r="B10" s="241" t="inlineStr">
+        <is>
+          <t>Scalar</t>
+        </is>
+      </c>
+      <c r="C10" s="242" t="n">
+        <v>157853559</v>
+      </c>
+      <c r="D10" s="243" t="n">
+        <v>2.549644</v>
+      </c>
+      <c r="E10" s="244" t="n">
+        <v>0.00870108</v>
+      </c>
+      <c r="F10" s="245" t="n">
+        <v>22.18465641552</v>
+      </c>
+      <c r="G10" s="245" t="n">
+        <v>0.3922116185632191</v>
+      </c>
+      <c r="H10" s="245" t="n">
+        <v>56.56297612189206</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="246" t="inlineStr">
+        <is>
+          <t>Controlled comparison at fixed sequence 256 (RVV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="233" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B11" s="233" t="inlineStr">
+      <c r="B13" s="233" t="inlineStr">
         <is>
           <t>d64_seq256</t>
         </is>
       </c>
-      <c r="C11" s="233" t="inlineStr">
+      <c r="C13" s="233" t="inlineStr">
         <is>
           <t>d108_seq256</t>
         </is>
       </c>
-      <c r="D11" s="233" t="inlineStr">
+      <c r="D13" s="233" t="inlineStr">
         <is>
           <t>d108 / d64</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="247" t="inlineStr">
-        <is>
-          <t>Committed instructions</t>
-        </is>
-      </c>
-      <c r="B12" s="242" t="n">
-        <v>6268591</v>
-      </c>
-      <c r="C12" s="242" t="n">
-        <v>19948310</v>
-      </c>
-      <c r="D12" s="248" t="n">
-        <v>3.182263765493713</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="247" t="inlineStr">
-        <is>
-          <t>Execution time (s)</t>
-        </is>
-      </c>
-      <c r="B13" s="243" t="n">
-        <v>0.08339000000000001</v>
-      </c>
-      <c r="C13" s="243" t="n">
-        <v>0.286467</v>
-      </c>
-      <c r="D13" s="248" t="n">
-        <v>3.435268017747931</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="247" t="inlineStr">
         <is>
-          <t>Energy per inference (mJ)</t>
-        </is>
-      </c>
-      <c r="B14" s="245" t="n">
-        <v>0.9312578250000001</v>
-      </c>
-      <c r="C14" s="245" t="n">
-        <v>3.009679595400001</v>
+          <t>Committed instructions</t>
+        </is>
+      </c>
+      <c r="B14" s="242" t="n">
+        <v>6275503</v>
+      </c>
+      <c r="C14" s="242" t="n">
+        <v>19948310</v>
       </c>
       <c r="D14" s="248" t="n">
-        <v>3.231843550307886</v>
+        <v>3.178758738542552</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="247" t="inlineStr">
         <is>
+          <t>Execution time (s)</t>
+        </is>
+      </c>
+      <c r="B15" s="243" t="n">
+        <v>0.086399</v>
+      </c>
+      <c r="C15" s="243" t="n">
+        <v>0.287988</v>
+      </c>
+      <c r="D15" s="248" t="n">
+        <v>3.333233023530365</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="247" t="inlineStr">
+        <is>
+          <t>Energy per inference (mJ)</t>
+        </is>
+      </c>
+      <c r="B16" s="245" t="n">
+        <v>0.8756797847000001</v>
+      </c>
+      <c r="C16" s="245" t="n">
+        <v>2.856806401440001</v>
+      </c>
+      <c r="D16" s="248" t="n">
+        <v>3.262387063575661</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="247" t="inlineStr">
+        <is>
           <t>Accuracy (PyTorch)</t>
         </is>
       </c>
-      <c r="B15" s="249" t="n">
+      <c r="B17" s="249" t="n">
         <v>0.796</v>
       </c>
-      <c r="C15" s="249" t="n">
+      <c r="C17" s="249" t="n">
         <v>0.8085</v>
       </c>
-      <c r="D15" s="250" t="n">
+      <c r="D17" s="250" t="n">
         <v>0.01249999999999996</v>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1" s="227">
-      <c r="A16" s="251" t="inlineStr">
-        <is>
-          <t>Reading: at a fixed 256 token sequence the larger model (108 wide, 3 layers) costs 3.2 times the instructions and 3.2 times the energy of the smaller (64 wide, 2 layers), for 1.25 points of accuracy. The earlier speed gap was the sequence length, not the width.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="246" t="inlineStr">
-        <is>
-          <t>RVV advantage at fixed sequence 256 (scalar divided by RVV)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="233" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B19" s="233" t="inlineStr">
-        <is>
-          <t>Fewer instructions</t>
-        </is>
-      </c>
-      <c r="C19" s="233" t="inlineStr">
-        <is>
-          <t>Faster (time)</t>
-        </is>
-      </c>
-      <c r="D19" s="233" t="inlineStr">
-        <is>
-          <t>Less energy</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="247" t="inlineStr">
-        <is>
-          <t>d64_seq256</t>
-        </is>
-      </c>
-      <c r="B20" s="248" t="n">
-        <v>1.990167008822238</v>
-      </c>
-      <c r="C20" s="248" t="n">
-        <v>2.415481472598633</v>
-      </c>
-      <c r="D20" s="248" t="n">
-        <v>2.073507263308096</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="247" t="inlineStr">
-        <is>
-          <t>d108_seq256</t>
-        </is>
-      </c>
-      <c r="B21" s="248" t="n">
-        <v>1.656964123777904</v>
-      </c>
-      <c r="C21" s="248" t="n">
-        <v>1.856932910247952</v>
-      </c>
-      <c r="D21" s="248" t="n">
-        <v>1.698612332460112</v>
+    <row r="18" ht="44" customHeight="1" s="227">
+      <c r="A18" s="251" t="inlineStr">
+        <is>
+          <t>Reading: at a fixed 256 token sequence the larger model costs 3.2 times the instructions and 3.3 times the energy of the smaller, for 1.25 points of accuracy. The earlier speed gap was the sequence length, not the width.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -34923,8 +34922,8 @@
     <row r="21"/>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A19:E21"/>
   </mergeCells>

</xml_diff>